<commit_message>
Update threat catalogue spreadsheet
</commit_message>
<xml_diff>
--- a/ThreatCatalogue/ICSThreatCatalogue (9).xlsx
+++ b/ThreatCatalogue/ICSThreatCatalogue (9).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielegranata/SystematicThreatSearchICS/ThreatCatalogue/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466EA90A-E447-6341-865D-DE3C03B0D6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC851EA-A633-E34D-A8B1-8C8130309E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3300" yWindow="-21100" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3300" yWindow="22480" windowWidth="36000" windowHeight="20880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Accepted Paper" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4607" uniqueCount="2790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4625" uniqueCount="2799">
   <si>
     <t>Column1</t>
   </si>
@@ -8415,6 +8415,33 @@
   </si>
   <si>
     <t>312, 313</t>
+  </si>
+  <si>
+    <t>94,151</t>
+  </si>
+  <si>
+    <t>272, 220</t>
+  </si>
+  <si>
+    <t>157, 118</t>
+  </si>
+  <si>
+    <t>159, 117, 169</t>
+  </si>
+  <si>
+    <t>584, 585</t>
+  </si>
+  <si>
+    <t>242, 151</t>
+  </si>
+  <si>
+    <t>66, 220, 272</t>
+  </si>
+  <si>
+    <t>115, 118</t>
+  </si>
+  <si>
+    <t>115, 151</t>
   </si>
 </sst>
 </file>
@@ -8565,7 +8592,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8620,8 +8647,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -8756,11 +8789,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF95B3D7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -8961,11 +9018,32 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="62">
+  <dxfs count="64">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -8990,382 +9068,25 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
+        <color rgb="FF9C0006"/>
       </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
+        <color rgb="FF9C0006"/>
       </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left/>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <name val="Calibri"/>
-        <scheme val="major"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color rgb="FF000000"/>
-        </vertical>
-        <horizontal style="thin">
-          <color rgb="FF000000"/>
-        </horizontal>
-      </border>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -10141,6 +9862,385 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left/>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Calibri"/>
+        <scheme val="major"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
@@ -10175,12 +10275,12 @@
   </dxfs>
   <tableStyles count="2">
     <tableStyle name="ThreatsPerAssetType-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="firstRowStripe" dxfId="63"/>
+      <tableStyleElement type="secondRowStripe" dxfId="62"/>
+    </tableStyle>
+    <tableStyle name="Asset Types-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="firstRowStripe" dxfId="61"/>
       <tableStyleElement type="secondRowStripe" dxfId="60"/>
-    </tableStyle>
-    <tableStyle name="Asset Types-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="firstRowStripe" dxfId="59"/>
-      <tableStyleElement type="secondRowStripe" dxfId="58"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -10195,79 +10295,79 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BE6C99E9-8D0F-4768-8A88-32E78696FCDF}" name="Table3" displayName="Table3" ref="A1:AX126" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BE6C99E9-8D0F-4768-8A88-32E78696FCDF}" name="Table3" displayName="Table3" ref="A1:AX126" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A1:AX126" xr:uid="{BE6C99E9-8D0F-4768-8A88-32E78696FCDF}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AX126">
     <sortCondition ref="A1:A126"/>
   </sortState>
   <tableColumns count="50">
-    <tableColumn id="2" xr3:uid="{92F25BBB-FDFC-4DF5-8410-EB7AC9797F46}" name="Column1" dataDxfId="55"/>
-    <tableColumn id="48" xr3:uid="{06F03740-0DBA-4157-96DB-81F9B556B719}" name="Download" dataDxfId="54"/>
-    <tableColumn id="49" xr3:uid="{9AB45D3F-BF1F-4CCC-8581-51FC7C72FB90}" name="Accepted" dataDxfId="53"/>
-    <tableColumn id="50" xr3:uid="{739D4D63-29BD-445D-9D0C-1F52A588262E}" name="Rejected" dataDxfId="52"/>
-    <tableColumn id="1" xr3:uid="{2FCDDDB1-6CF9-4D0C-8A71-1D1228DD5697}" name="In reference" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{B69423CD-CE76-466C-843C-455FF0166329}" name="﻿&quot;Authors&quot;" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{26E3A757-F3E5-44E5-99A7-A22AEF8713AC}" name="Author full names" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{CB43E959-836A-4AF5-B915-131294407B67}" name="Author(s) ID" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{0EEFE55B-5D1A-4059-B57D-BA21DF853176}" name="Title" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{3E2232A3-6CFC-400B-A09E-E74405D4D49B}" name="Year" dataDxfId="46"/>
-    <tableColumn id="8" xr3:uid="{8E573524-26CF-48B4-9D6D-C3405FD90F77}" name="Source title" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{88AF7DE8-89F5-40EA-ADAB-881C9BE16750}" name="Volume" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{C02E9D01-35A0-4916-A8BC-3D19F32989E5}" name="Issue" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{92F25BBB-FDFC-4DF5-8410-EB7AC9797F46}" name="Column1" dataDxfId="44"/>
+    <tableColumn id="48" xr3:uid="{06F03740-0DBA-4157-96DB-81F9B556B719}" name="Download" dataDxfId="43"/>
+    <tableColumn id="49" xr3:uid="{9AB45D3F-BF1F-4CCC-8581-51FC7C72FB90}" name="Accepted" dataDxfId="42"/>
+    <tableColumn id="50" xr3:uid="{739D4D63-29BD-445D-9D0C-1F52A588262E}" name="Rejected" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{2FCDDDB1-6CF9-4D0C-8A71-1D1228DD5697}" name="In reference" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{B69423CD-CE76-466C-843C-455FF0166329}" name="﻿&quot;Authors&quot;" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{26E3A757-F3E5-44E5-99A7-A22AEF8713AC}" name="Author full names" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{CB43E959-836A-4AF5-B915-131294407B67}" name="Author(s) ID" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{0EEFE55B-5D1A-4059-B57D-BA21DF853176}" name="Title" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{3E2232A3-6CFC-400B-A09E-E74405D4D49B}" name="Year" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{8E573524-26CF-48B4-9D6D-C3405FD90F77}" name="Source title" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{88AF7DE8-89F5-40EA-ADAB-881C9BE16750}" name="Volume" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{C02E9D01-35A0-4916-A8BC-3D19F32989E5}" name="Issue" dataDxfId="32"/>
     <tableColumn id="11" xr3:uid="{4F3DEF62-75B0-4908-93F2-3E7F0CA7B506}" name="Art. No."/>
-    <tableColumn id="12" xr3:uid="{F4C7E935-4D8E-479C-ADF0-2A68273DDF3A}" name="Page start" dataDxfId="42"/>
-    <tableColumn id="13" xr3:uid="{3A0180AF-D667-4EBB-84D2-BE70D2A8C5AB}" name="Page end" dataDxfId="41"/>
-    <tableColumn id="14" xr3:uid="{3E747361-8302-41FE-A7EA-E4390370502B}" name="Page count" dataDxfId="40"/>
-    <tableColumn id="15" xr3:uid="{86D187D6-9C0B-4011-BDEA-3FD57DBF6030}" name="Cited by" dataDxfId="39"/>
-    <tableColumn id="16" xr3:uid="{60778912-CE9B-4D27-906E-C5FC4DC35848}" name="DOI" dataDxfId="38"/>
-    <tableColumn id="17" xr3:uid="{E8A489B1-A6E1-42F0-8FF5-BC78D1934DC8}" name="Link" dataDxfId="37"/>
-    <tableColumn id="18" xr3:uid="{D8D0AAEC-EF06-4A21-AD21-22DFFC39CBC4}" name="Affiliations" dataDxfId="36"/>
-    <tableColumn id="19" xr3:uid="{01104F93-0B98-4C16-9F34-DA548FC20E7B}" name="Authors with affiliations" dataDxfId="35"/>
-    <tableColumn id="20" xr3:uid="{4E0BA5E4-4BA0-446F-A68B-E9D56A0B8C5D}" name="Abstract" dataDxfId="34"/>
-    <tableColumn id="21" xr3:uid="{F2653DA4-9FD0-4568-B8FA-9E10F3BCDC7B}" name="Author Keywords" dataDxfId="33"/>
-    <tableColumn id="22" xr3:uid="{D2249547-3682-443A-B4BA-E592229138A8}" name="Index Keywords" dataDxfId="32"/>
-    <tableColumn id="23" xr3:uid="{6E298AAB-8D6D-4087-9ECB-D8883E1525A2}" name="Correspondence Address" dataDxfId="31"/>
+    <tableColumn id="12" xr3:uid="{F4C7E935-4D8E-479C-ADF0-2A68273DDF3A}" name="Page start" dataDxfId="31"/>
+    <tableColumn id="13" xr3:uid="{3A0180AF-D667-4EBB-84D2-BE70D2A8C5AB}" name="Page end" dataDxfId="30"/>
+    <tableColumn id="14" xr3:uid="{3E747361-8302-41FE-A7EA-E4390370502B}" name="Page count" dataDxfId="29"/>
+    <tableColumn id="15" xr3:uid="{86D187D6-9C0B-4011-BDEA-3FD57DBF6030}" name="Cited by" dataDxfId="28"/>
+    <tableColumn id="16" xr3:uid="{60778912-CE9B-4D27-906E-C5FC4DC35848}" name="DOI" dataDxfId="27"/>
+    <tableColumn id="17" xr3:uid="{E8A489B1-A6E1-42F0-8FF5-BC78D1934DC8}" name="Link" dataDxfId="26"/>
+    <tableColumn id="18" xr3:uid="{D8D0AAEC-EF06-4A21-AD21-22DFFC39CBC4}" name="Affiliations" dataDxfId="25"/>
+    <tableColumn id="19" xr3:uid="{01104F93-0B98-4C16-9F34-DA548FC20E7B}" name="Authors with affiliations" dataDxfId="24"/>
+    <tableColumn id="20" xr3:uid="{4E0BA5E4-4BA0-446F-A68B-E9D56A0B8C5D}" name="Abstract" dataDxfId="23"/>
+    <tableColumn id="21" xr3:uid="{F2653DA4-9FD0-4568-B8FA-9E10F3BCDC7B}" name="Author Keywords" dataDxfId="22"/>
+    <tableColumn id="22" xr3:uid="{D2249547-3682-443A-B4BA-E592229138A8}" name="Index Keywords" dataDxfId="21"/>
+    <tableColumn id="23" xr3:uid="{6E298AAB-8D6D-4087-9ECB-D8883E1525A2}" name="Correspondence Address" dataDxfId="20"/>
     <tableColumn id="24" xr3:uid="{D1EB0EA7-FE31-4B20-AE65-B2392C3BBAED}" name="Editors"/>
-    <tableColumn id="25" xr3:uid="{2CB62BBB-6DBD-4A1E-B736-B578684E2BF6}" name="Publisher" dataDxfId="30"/>
-    <tableColumn id="26" xr3:uid="{67560EDC-8213-48CE-B48D-7C437F0D9804}" name="ISSN" dataDxfId="29"/>
+    <tableColumn id="25" xr3:uid="{2CB62BBB-6DBD-4A1E-B736-B578684E2BF6}" name="Publisher" dataDxfId="19"/>
+    <tableColumn id="26" xr3:uid="{67560EDC-8213-48CE-B48D-7C437F0D9804}" name="ISSN" dataDxfId="18"/>
     <tableColumn id="27" xr3:uid="{3291DB44-2324-480C-AAA6-EB68F9F87BB7}" name="ISBN"/>
     <tableColumn id="28" xr3:uid="{36E6C0E8-57C7-457A-A892-E9F456C42932}" name="CODEN"/>
     <tableColumn id="29" xr3:uid="{95E818E6-CF8A-4598-8D9D-0C0E7B403ACD}" name="PubMed ID"/>
-    <tableColumn id="30" xr3:uid="{F5038767-AF55-4004-AA7C-FD5ABCF2E258}" name="Language of Original Document" dataDxfId="28"/>
-    <tableColumn id="31" xr3:uid="{7BC1B7CF-1FEA-4EF4-890A-CB5E5A2A992F}" name="Abbreviated Source Title" dataDxfId="27"/>
-    <tableColumn id="32" xr3:uid="{64B515DB-469D-4008-8E6A-7EE6956B9560}" name="Document Type" dataDxfId="26"/>
-    <tableColumn id="33" xr3:uid="{B3E72E21-7F24-4629-84C2-B5EAFD1E1AD3}" name="Publication Stage" dataDxfId="25"/>
+    <tableColumn id="30" xr3:uid="{F5038767-AF55-4004-AA7C-FD5ABCF2E258}" name="Language of Original Document" dataDxfId="17"/>
+    <tableColumn id="31" xr3:uid="{7BC1B7CF-1FEA-4EF4-890A-CB5E5A2A992F}" name="Abbreviated Source Title" dataDxfId="16"/>
+    <tableColumn id="32" xr3:uid="{64B515DB-469D-4008-8E6A-7EE6956B9560}" name="Document Type" dataDxfId="15"/>
+    <tableColumn id="33" xr3:uid="{B3E72E21-7F24-4629-84C2-B5EAFD1E1AD3}" name="Publication Stage" dataDxfId="14"/>
     <tableColumn id="34" xr3:uid="{03ABA5E7-3FE2-4978-AFEF-6683932884E8}" name="Open Access"/>
-    <tableColumn id="35" xr3:uid="{60A42EB9-C494-4A09-BA6A-A47D10DDF8DD}" name="Source" dataDxfId="24"/>
-    <tableColumn id="36" xr3:uid="{D8FF8184-568F-42B1-A938-C515B8E914FA}" name="EID" dataDxfId="23"/>
-    <tableColumn id="37" xr3:uid="{CF5BBE77-3920-46DD-A33D-A3412BB21CDE}" name="asreview_label" dataDxfId="22"/>
-    <tableColumn id="38" xr3:uid="{2FED1A7F-FD1E-486D-8D03-97FD16861F19}" name="asreview_time" dataDxfId="21"/>
+    <tableColumn id="35" xr3:uid="{60A42EB9-C494-4A09-BA6A-A47D10DDF8DD}" name="Source" dataDxfId="13"/>
+    <tableColumn id="36" xr3:uid="{D8FF8184-568F-42B1-A938-C515B8E914FA}" name="EID" dataDxfId="12"/>
+    <tableColumn id="37" xr3:uid="{CF5BBE77-3920-46DD-A33D-A3412BB21CDE}" name="asreview_label" dataDxfId="11"/>
+    <tableColumn id="38" xr3:uid="{2FED1A7F-FD1E-486D-8D03-97FD16861F19}" name="asreview_time" dataDxfId="10"/>
     <tableColumn id="39" xr3:uid="{74177341-EF22-4B90-B133-29CF084A47D6}" name="asreview_note"/>
     <tableColumn id="40" xr3:uid="{876E2CD9-1FBE-457D-B69C-9EFD327CE7B3}" name="asreview_tag_inclusion_threatanalysis"/>
     <tableColumn id="41" xr3:uid="{184251F7-B449-4E59-AA54-E3448627EA86}" name="asreview_tag_inclusion_containsthreats"/>
-    <tableColumn id="42" xr3:uid="{439445E7-6353-4BA1-92A5-7C1C052100ED}" name="asreview_tag_exclusion_not_relatedtoics" dataDxfId="20"/>
-    <tableColumn id="43" xr3:uid="{A1761CEC-C511-4ECC-9493-63BEBAB024E6}" name="asreview_tag_exclusion_notthreatmodelling" dataDxfId="19"/>
-    <tableColumn id="44" xr3:uid="{610CC079-5339-4576-B53A-B40B0EE707E4}" name="asreview_tag_exclusion_notwritterinenglish" dataDxfId="18"/>
-    <tableColumn id="45" xr3:uid="{A1A5AEEA-8644-43C2-B8E9-7F97F260EDBD}" name="asreview_tag_exclusion_nottechnical" dataDxfId="17"/>
-    <tableColumn id="46" xr3:uid="{6F9B9F94-5E93-4439-A4AE-45A7FF622ED0}" name="asreview_tag_inclusion_threatanalysismethodology" dataDxfId="16"/>
-    <tableColumn id="47" xr3:uid="{30792347-2530-444A-B105-9270AC5016BF}" name="asreview_tag_inclusion_containsthreats_non_threat_models" dataDxfId="15"/>
+    <tableColumn id="42" xr3:uid="{439445E7-6353-4BA1-92A5-7C1C052100ED}" name="asreview_tag_exclusion_not_relatedtoics" dataDxfId="9"/>
+    <tableColumn id="43" xr3:uid="{A1761CEC-C511-4ECC-9493-63BEBAB024E6}" name="asreview_tag_exclusion_notthreatmodelling" dataDxfId="8"/>
+    <tableColumn id="44" xr3:uid="{610CC079-5339-4576-B53A-B40B0EE707E4}" name="asreview_tag_exclusion_notwritterinenglish" dataDxfId="7"/>
+    <tableColumn id="45" xr3:uid="{A1A5AEEA-8644-43C2-B8E9-7F97F260EDBD}" name="asreview_tag_exclusion_nottechnical" dataDxfId="6"/>
+    <tableColumn id="46" xr3:uid="{6F9B9F94-5E93-4439-A4AE-45A7FF622ED0}" name="asreview_tag_inclusion_threatanalysismethodology" dataDxfId="5"/>
+    <tableColumn id="47" xr3:uid="{30792347-2530-444A-B105-9270AC5016BF}" name="asreview_tag_inclusion_containsthreats_non_threat_models" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B2:J50" headerRowCount="0" headerRowDxfId="14" dataDxfId="13" totalsRowDxfId="11" tableBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B2:J50" headerRowCount="0" headerRowDxfId="59" dataDxfId="58" totalsRowDxfId="56" tableBorderDxfId="57">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{7BE39368-27BE-4152-B500-D446A6F7FA0E}" name="Colonna1" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{5E191DFD-2D16-4F95-A622-E074F7EE438C}" name="Colonna2" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{0B58A523-8139-4ABC-BE62-A2F4CE2629E0}" name="Colonna3" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{C557E0D8-FF14-4B07-8A1D-A76E7C101036}" name="Colonna4" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{37E34D9C-145E-41F5-BF78-14B521E4D34E}" name="Colonna5" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{B23C818F-B55B-4868-AB92-C8649F17F801}" name="Colonna6" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{94F30ACB-7852-44F7-8CAA-EC0AFFF5ECEE}" name="Colonna7" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{7BE39368-27BE-4152-B500-D446A6F7FA0E}" name="Colonna1" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{5E191DFD-2D16-4F95-A622-E074F7EE438C}" name="Colonna2" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{0B58A523-8139-4ABC-BE62-A2F4CE2629E0}" name="Colonna3" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{C557E0D8-FF14-4B07-8A1D-A76E7C101036}" name="Colonna4" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{37E34D9C-145E-41F5-BF78-14B521E4D34E}" name="Colonna5" dataDxfId="49"/>
+    <tableColumn id="8" xr3:uid="{B23C818F-B55B-4868-AB92-C8649F17F801}" name="Colonna6" dataDxfId="48"/>
+    <tableColumn id="9" xr3:uid="{94F30ACB-7852-44F7-8CAA-EC0AFFF5ECEE}" name="Colonna7" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="ThreatsPerAssetType-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -29910,12 +30010,12 @@
     <row r="1008" ht="15.75" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="O1:R1">
-    <cfRule type="containsBlanks" dxfId="1" priority="2" stopIfTrue="1">
+    <cfRule type="containsBlanks" dxfId="3" priority="2" stopIfTrue="1">
       <formula>LEN(TRIM(O1))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:R2">
-    <cfRule type="containsBlanks" dxfId="0" priority="1" stopIfTrue="1">
+    <cfRule type="containsBlanks" dxfId="2" priority="1" stopIfTrue="1">
       <formula>LEN(TRIM(P2))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -29929,7 +30029,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P999"/>
+  <dimension ref="A1:T999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="8" customWidth="1"/>
@@ -29942,13 +30042,14 @@
     <col min="10" max="12" width="10.6640625" style="8" customWidth="1"/>
     <col min="13" max="13" width="16.5" style="8" customWidth="1"/>
     <col min="14" max="14" width="17" style="8" customWidth="1"/>
-    <col min="15" max="15" width="10.6640625" style="8" customWidth="1"/>
-    <col min="16" max="16" width="21" style="8" customWidth="1"/>
-    <col min="17" max="26" width="10.6640625" style="8" customWidth="1"/>
+    <col min="15" max="15" width="13.1640625" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="13.1640625" customWidth="1"/>
+    <col min="18" max="26" width="10.6640625" style="8" customWidth="1"/>
     <col min="27" max="16384" width="14.5" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="24.75" customHeight="1">
+    <row r="1" spans="1:20" ht="24.75" customHeight="1">
       <c r="A1" s="18" t="s">
         <v>2465</v>
       </c>
@@ -29991,9 +30092,17 @@
       <c r="N1" s="18" t="s">
         <v>2302</v>
       </c>
-      <c r="O1" s="45"/>
-    </row>
-    <row r="2" spans="1:16" ht="72.75" customHeight="1">
+      <c r="O1" s="95" t="s">
+        <v>2303</v>
+      </c>
+      <c r="P1" s="95" t="s">
+        <v>2304</v>
+      </c>
+      <c r="Q1" s="95" t="s">
+        <v>2305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="72.75" customHeight="1">
       <c r="A2" s="46" t="s">
         <v>2467</v>
       </c>
@@ -30035,15 +30144,21 @@
         <f t="shared" ref="M2:M48" si="1">CONCATENATE("[",J2,",",K2,",",L2,"]")</f>
         <v>[f,p,p]</v>
       </c>
-      <c r="N2" s="82" t="s">
+      <c r="N2" s="92" t="s">
         <v>2471</v>
       </c>
-      <c r="O2" s="45"/>
-      <c r="P2" s="8" t="s">
+      <c r="O2" s="100" t="s">
+        <v>2790</v>
+      </c>
+      <c r="P2" s="100" t="s">
+        <v>2791</v>
+      </c>
+      <c r="Q2" s="96"/>
+      <c r="T2" s="8" t="s">
         <v>2472</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="57" customHeight="1">
+    <row r="3" spans="1:20" ht="57" customHeight="1">
       <c r="A3" s="46" t="s">
         <v>2467</v>
       </c>
@@ -30085,12 +30200,20 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N3" s="83" t="s">
+      <c r="N3" s="93" t="s">
         <v>2476</v>
       </c>
-      <c r="O3" s="45"/>
-    </row>
-    <row r="4" spans="1:16" ht="60.75" customHeight="1">
+      <c r="O3" s="98" t="s">
+        <v>2792</v>
+      </c>
+      <c r="P3" s="98" t="s">
+        <v>2793</v>
+      </c>
+      <c r="Q3" s="98" t="s">
+        <v>2794</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="60.75" customHeight="1">
       <c r="A4" s="46" t="s">
         <v>2467</v>
       </c>
@@ -30132,12 +30255,18 @@
         <f t="shared" si="1"/>
         <v>[n,n,p]</v>
       </c>
-      <c r="N4" s="82" t="s">
+      <c r="N4" s="92" t="s">
         <v>2480</v>
       </c>
-      <c r="O4" s="45"/>
-    </row>
-    <row r="5" spans="1:16" ht="60" customHeight="1">
+      <c r="O4" s="98">
+        <v>125</v>
+      </c>
+      <c r="P4" s="98">
+        <v>488</v>
+      </c>
+      <c r="Q4" s="97"/>
+    </row>
+    <row r="5" spans="1:20" ht="60" customHeight="1">
       <c r="A5" s="46" t="s">
         <v>2467</v>
       </c>
@@ -30179,12 +30308,18 @@
         <f t="shared" si="1"/>
         <v>[p,p,p]</v>
       </c>
-      <c r="N5" s="47" t="s">
+      <c r="N5" s="94" t="s">
         <v>2482</v>
       </c>
-      <c r="O5" s="45"/>
-    </row>
-    <row r="6" spans="1:16" ht="57" customHeight="1">
+      <c r="O5" s="98" t="s">
+        <v>2795</v>
+      </c>
+      <c r="P5" s="98" t="s">
+        <v>2796</v>
+      </c>
+      <c r="Q5" s="97"/>
+    </row>
+    <row r="6" spans="1:20" ht="57" customHeight="1">
       <c r="A6" s="46" t="s">
         <v>2467</v>
       </c>
@@ -30226,12 +30361,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N6" s="82" t="s">
+      <c r="N6" s="92" t="s">
         <v>2485</v>
       </c>
-      <c r="O6" s="45"/>
-    </row>
-    <row r="7" spans="1:16" ht="64">
+      <c r="O6" s="97">
+        <v>115</v>
+      </c>
+      <c r="P6" s="97">
+        <v>203</v>
+      </c>
+      <c r="Q6" s="97"/>
+    </row>
+    <row r="7" spans="1:20" ht="64">
       <c r="A7" s="46" t="s">
         <v>2467</v>
       </c>
@@ -30273,12 +30414,18 @@
         <f t="shared" si="1"/>
         <v>[f,n,n]</v>
       </c>
-      <c r="N7" s="47">
+      <c r="N7" s="94">
         <v>844</v>
       </c>
-      <c r="O7" s="45"/>
-    </row>
-    <row r="8" spans="1:16" ht="70.5" customHeight="1">
+      <c r="O7" s="98" t="s">
+        <v>2792</v>
+      </c>
+      <c r="P7" s="97">
+        <v>117</v>
+      </c>
+      <c r="Q7" s="97"/>
+    </row>
+    <row r="8" spans="1:20" ht="70.5" customHeight="1">
       <c r="A8" s="47" t="s">
         <v>2488</v>
       </c>
@@ -30320,12 +30467,16 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N8" s="47">
+      <c r="N8" s="94">
         <v>308</v>
       </c>
-      <c r="O8" s="45"/>
-    </row>
-    <row r="9" spans="1:16" ht="64">
+      <c r="O8" s="97">
+        <v>115</v>
+      </c>
+      <c r="P8" s="97"/>
+      <c r="Q8" s="97"/>
+    </row>
+    <row r="9" spans="1:20" ht="64">
       <c r="A9" s="47" t="s">
         <v>2488</v>
       </c>
@@ -30367,12 +30518,18 @@
         <f t="shared" si="1"/>
         <v>[p,p,n]</v>
       </c>
-      <c r="N9" s="47" t="s">
+      <c r="N9" s="94" t="s">
         <v>2492</v>
       </c>
-      <c r="O9" s="45"/>
-    </row>
-    <row r="10" spans="1:16" ht="80">
+      <c r="O9" s="98">
+        <v>151</v>
+      </c>
+      <c r="P9" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q9" s="97"/>
+    </row>
+    <row r="10" spans="1:20" ht="80">
       <c r="A10" s="47" t="s">
         <v>2488</v>
       </c>
@@ -30414,12 +30571,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N10" s="47" t="s">
+      <c r="N10" s="94" t="s">
         <v>2495</v>
       </c>
-      <c r="O10" s="45"/>
-    </row>
-    <row r="11" spans="1:16" ht="51.75" customHeight="1">
+      <c r="O10" s="98">
+        <v>242</v>
+      </c>
+      <c r="P10" s="98">
+        <v>272</v>
+      </c>
+      <c r="Q10" s="97"/>
+    </row>
+    <row r="11" spans="1:20" ht="51.75" customHeight="1">
       <c r="A11" s="47" t="s">
         <v>2488</v>
       </c>
@@ -30461,12 +30624,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N11" s="83" t="s">
+      <c r="N11" s="93" t="s">
         <v>2496</v>
       </c>
-      <c r="O11" s="45"/>
-    </row>
-    <row r="12" spans="1:16" ht="42.75" customHeight="1">
+      <c r="O11" s="98" t="s">
+        <v>2792</v>
+      </c>
+      <c r="P11" s="97">
+        <v>117</v>
+      </c>
+      <c r="Q11" s="97"/>
+    </row>
+    <row r="12" spans="1:20" ht="42.75" customHeight="1">
       <c r="A12" s="47" t="s">
         <v>2497</v>
       </c>
@@ -30508,12 +30677,16 @@
         <f t="shared" si="1"/>
         <v>[f,n,n]</v>
       </c>
-      <c r="N12" s="47">
+      <c r="N12" s="94">
         <v>652</v>
       </c>
-      <c r="O12" s="45"/>
-    </row>
-    <row r="13" spans="1:16" ht="38.25" customHeight="1">
+      <c r="O12" s="98" t="s">
+        <v>2797</v>
+      </c>
+      <c r="P12" s="97"/>
+      <c r="Q12" s="97"/>
+    </row>
+    <row r="13" spans="1:20" ht="38.25" customHeight="1">
       <c r="A13" s="47" t="s">
         <v>2497</v>
       </c>
@@ -30555,12 +30728,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,n]</v>
       </c>
-      <c r="N13" s="47">
+      <c r="N13" s="94">
         <v>652</v>
       </c>
-      <c r="O13" s="45"/>
-    </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1">
+      <c r="O13" s="98">
+        <v>151</v>
+      </c>
+      <c r="P13" s="98">
+        <v>272</v>
+      </c>
+      <c r="Q13" s="97"/>
+    </row>
+    <row r="14" spans="1:20" ht="15" customHeight="1">
       <c r="A14" s="47" t="s">
         <v>2497</v>
       </c>
@@ -30602,12 +30781,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,n]</v>
       </c>
-      <c r="N14" s="47">
+      <c r="N14" s="94">
         <v>652</v>
       </c>
-      <c r="O14" s="45"/>
-    </row>
-    <row r="15" spans="1:16" ht="59.25" customHeight="1">
+      <c r="O14" s="97">
+        <v>94</v>
+      </c>
+      <c r="P14" s="98">
+        <v>21</v>
+      </c>
+      <c r="Q14" s="97"/>
+    </row>
+    <row r="15" spans="1:20" ht="59.25" customHeight="1">
       <c r="A15" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30649,12 +30834,16 @@
         <f t="shared" si="1"/>
         <v>[n,n,f]</v>
       </c>
-      <c r="N15" s="47" t="s">
+      <c r="N15" s="94" t="s">
         <v>2508</v>
       </c>
-      <c r="O15" s="45"/>
-    </row>
-    <row r="16" spans="1:16" ht="58.5" customHeight="1">
+      <c r="O15" s="97">
+        <v>125</v>
+      </c>
+      <c r="P15" s="97"/>
+      <c r="Q15" s="97"/>
+    </row>
+    <row r="16" spans="1:20" ht="58.5" customHeight="1">
       <c r="A16" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30696,12 +30885,16 @@
         <f t="shared" si="1"/>
         <v>[f,f,n]</v>
       </c>
-      <c r="N16" s="47" t="s">
+      <c r="N16" s="94" t="s">
         <v>2508</v>
       </c>
-      <c r="O16" s="45"/>
-    </row>
-    <row r="17" spans="1:15" ht="45.75" customHeight="1">
+      <c r="O16" s="97">
+        <v>115</v>
+      </c>
+      <c r="P16" s="97"/>
+      <c r="Q16" s="97"/>
+    </row>
+    <row r="17" spans="1:17" ht="45.75" customHeight="1">
       <c r="A17" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30743,12 +30936,16 @@
         <f t="shared" si="1"/>
         <v>[n,f,f]</v>
       </c>
-      <c r="N17" s="47">
+      <c r="N17" s="94">
         <v>570</v>
       </c>
-      <c r="O17" s="45"/>
-    </row>
-    <row r="18" spans="1:15" ht="45.75" customHeight="1">
+      <c r="O17" s="97">
+        <v>20</v>
+      </c>
+      <c r="P17" s="97"/>
+      <c r="Q17" s="97"/>
+    </row>
+    <row r="18" spans="1:17" ht="45.75" customHeight="1">
       <c r="A18" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30790,12 +30987,16 @@
         <f t="shared" si="1"/>
         <v>[n,f,f]</v>
       </c>
-      <c r="N18" s="47" t="s">
+      <c r="N18" s="94" t="s">
         <v>2517</v>
       </c>
-      <c r="O18" s="45"/>
-    </row>
-    <row r="19" spans="1:15" ht="45.75" customHeight="1">
+      <c r="O18" s="97">
+        <v>115</v>
+      </c>
+      <c r="P18" s="98"/>
+      <c r="Q18" s="97"/>
+    </row>
+    <row r="19" spans="1:17" ht="45.75" customHeight="1">
       <c r="A19" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30837,12 +31038,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,p]</v>
       </c>
-      <c r="N19" s="47">
+      <c r="N19" s="94">
         <v>844</v>
       </c>
-      <c r="O19" s="45"/>
-    </row>
-    <row r="20" spans="1:15" ht="45.75" customHeight="1">
+      <c r="O19" s="97">
+        <v>151</v>
+      </c>
+      <c r="P19" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q19" s="97"/>
+    </row>
+    <row r="20" spans="1:17" ht="45.75" customHeight="1">
       <c r="A20" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30884,12 +31091,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,n]</v>
       </c>
-      <c r="N20" s="47">
+      <c r="N20" s="94">
         <v>844</v>
       </c>
-      <c r="O20" s="45"/>
-    </row>
-    <row r="21" spans="1:15" ht="45.75" customHeight="1">
+      <c r="O20" s="97">
+        <v>151</v>
+      </c>
+      <c r="P20" s="97">
+        <v>294</v>
+      </c>
+      <c r="Q20" s="97"/>
+    </row>
+    <row r="21" spans="1:17" ht="45.75" customHeight="1">
       <c r="A21" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30931,12 +31144,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,p]</v>
       </c>
-      <c r="N21" s="47">
+      <c r="N21" s="94">
         <v>870.22</v>
       </c>
-      <c r="O21" s="45"/>
-    </row>
-    <row r="22" spans="1:15" ht="45.75" customHeight="1">
+      <c r="O21" s="98">
+        <v>125</v>
+      </c>
+      <c r="P21" s="97">
+        <v>488</v>
+      </c>
+      <c r="Q21" s="99"/>
+    </row>
+    <row r="22" spans="1:17" ht="45.75" customHeight="1">
       <c r="A22" s="47" t="s">
         <v>2505</v>
       </c>
@@ -30978,12 +31197,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,n]</v>
       </c>
-      <c r="N22" s="47">
+      <c r="N22" s="94">
         <v>870</v>
       </c>
-      <c r="O22" s="45"/>
-    </row>
-    <row r="23" spans="1:15" ht="62.25" customHeight="1">
+      <c r="O22" s="98" t="s">
+        <v>2792</v>
+      </c>
+      <c r="P22" s="98">
+        <v>117</v>
+      </c>
+      <c r="Q22" s="99"/>
+    </row>
+    <row r="23" spans="1:17" ht="62.25" customHeight="1">
       <c r="A23" s="47" t="s">
         <v>2505</v>
       </c>
@@ -31025,12 +31250,16 @@
         <f t="shared" si="1"/>
         <v>[n,n,f]</v>
       </c>
-      <c r="N23" s="47">
+      <c r="N23" s="94">
         <v>884</v>
       </c>
-      <c r="O23" s="45"/>
-    </row>
-    <row r="24" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O23" s="98">
+        <v>20</v>
+      </c>
+      <c r="P23" s="98"/>
+      <c r="Q23" s="99"/>
+    </row>
+    <row r="24" spans="1:17" ht="42.75" customHeight="1">
       <c r="A24" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31072,12 +31301,16 @@
         <f t="shared" si="1"/>
         <v>[f,f,p]</v>
       </c>
-      <c r="N24" s="47" t="s">
+      <c r="N24" s="94" t="s">
         <v>2517</v>
       </c>
-      <c r="O24" s="45"/>
-    </row>
-    <row r="25" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O24" s="98">
+        <v>115</v>
+      </c>
+      <c r="P24" s="97"/>
+      <c r="Q24" s="99"/>
+    </row>
+    <row r="25" spans="1:17" ht="42.75" customHeight="1">
       <c r="A25" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31119,12 +31352,16 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N25" s="47" t="s">
+      <c r="N25" s="94" t="s">
         <v>2537</v>
       </c>
-      <c r="O25" s="45"/>
-    </row>
-    <row r="26" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O25" s="98">
+        <v>118</v>
+      </c>
+      <c r="P25" s="98"/>
+      <c r="Q25" s="99"/>
+    </row>
+    <row r="26" spans="1:17" ht="42.75" customHeight="1">
       <c r="A26" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31166,12 +31403,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N26" s="47">
+      <c r="N26" s="94">
         <v>722</v>
       </c>
-      <c r="O26" s="45"/>
-    </row>
-    <row r="27" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O26" s="98" t="s">
+        <v>2798</v>
+      </c>
+      <c r="P26" s="98">
+        <v>272</v>
+      </c>
+      <c r="Q26" s="99"/>
+    </row>
+    <row r="27" spans="1:17" ht="42.75" customHeight="1">
       <c r="A27" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31213,12 +31456,16 @@
         <f t="shared" si="1"/>
         <v>[n,n,p]</v>
       </c>
-      <c r="N27" s="47">
+      <c r="N27" s="94">
         <v>722</v>
       </c>
-      <c r="O27" s="45"/>
-    </row>
-    <row r="28" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O27" s="98">
+        <v>125</v>
+      </c>
+      <c r="P27" s="97"/>
+      <c r="Q27" s="99"/>
+    </row>
+    <row r="28" spans="1:17" ht="42.75" customHeight="1">
       <c r="A28" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31260,12 +31507,18 @@
         <f t="shared" si="1"/>
         <v>[p,p,n]</v>
       </c>
-      <c r="N28" s="47" t="s">
+      <c r="N28" s="94" t="s">
         <v>2544</v>
       </c>
-      <c r="O28" s="45"/>
-    </row>
-    <row r="29" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O28" s="97">
+        <v>157</v>
+      </c>
+      <c r="P28" s="97">
+        <v>118</v>
+      </c>
+      <c r="Q28" s="99"/>
+    </row>
+    <row r="29" spans="1:17" ht="42.75" customHeight="1">
       <c r="A29" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31307,12 +31560,16 @@
         <f t="shared" si="1"/>
         <v>[n,p,n]</v>
       </c>
-      <c r="N29" s="47" t="s">
+      <c r="N29" s="94" t="s">
         <v>2547</v>
       </c>
-      <c r="O29" s="45"/>
-    </row>
-    <row r="30" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O29" s="97">
+        <v>117</v>
+      </c>
+      <c r="P29" s="97"/>
+      <c r="Q29" s="99"/>
+    </row>
+    <row r="30" spans="1:17" ht="42.75" customHeight="1">
       <c r="A30" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31354,12 +31611,18 @@
         <f t="shared" si="1"/>
         <v>[n,n,p]</v>
       </c>
-      <c r="N30" s="47">
+      <c r="N30" s="94">
         <v>882</v>
       </c>
-      <c r="O30" s="45"/>
-    </row>
-    <row r="31" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O30" s="97">
+        <v>151</v>
+      </c>
+      <c r="P30" s="98">
+        <v>272</v>
+      </c>
+      <c r="Q30" s="99"/>
+    </row>
+    <row r="31" spans="1:17" ht="42.75" customHeight="1">
       <c r="A31" s="47" t="s">
         <v>2532</v>
       </c>
@@ -31401,12 +31664,16 @@
         <f t="shared" si="1"/>
         <v>[p,p,n]</v>
       </c>
-      <c r="N31" s="47">
+      <c r="N31" s="94">
         <v>882</v>
       </c>
-      <c r="O31" s="45"/>
-    </row>
-    <row r="32" spans="1:15" ht="49.5" customHeight="1">
+      <c r="O31" s="97">
+        <v>151</v>
+      </c>
+      <c r="P31" s="97"/>
+      <c r="Q31" s="99"/>
+    </row>
+    <row r="32" spans="1:17" ht="49.5" customHeight="1">
       <c r="A32" s="47" t="s">
         <v>2553</v>
       </c>
@@ -31448,12 +31715,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N32" s="47">
+      <c r="N32" s="94">
         <v>450</v>
       </c>
-      <c r="O32" s="45"/>
-    </row>
-    <row r="33" spans="1:15" ht="55.5" customHeight="1">
+      <c r="O32" s="97">
+        <v>118</v>
+      </c>
+      <c r="P32" s="97">
+        <v>117</v>
+      </c>
+      <c r="Q32" s="99"/>
+    </row>
+    <row r="33" spans="1:17" ht="55.5" customHeight="1">
       <c r="A33" s="47" t="s">
         <v>2556</v>
       </c>
@@ -31495,12 +31768,14 @@
         <f t="shared" si="1"/>
         <v>[n,n,f]</v>
       </c>
-      <c r="N33" s="47">
+      <c r="N33" s="94">
         <v>448</v>
       </c>
-      <c r="O33" s="45"/>
-    </row>
-    <row r="34" spans="1:15" ht="55.5" customHeight="1">
+      <c r="O33" s="101"/>
+      <c r="P33" s="101"/>
+      <c r="Q33" s="102"/>
+    </row>
+    <row r="34" spans="1:17" ht="55.5" customHeight="1">
       <c r="A34" s="47" t="s">
         <v>2559</v>
       </c>
@@ -31542,12 +31817,16 @@
         <f t="shared" si="1"/>
         <v>[f,p,n]</v>
       </c>
-      <c r="N34" s="47">
+      <c r="N34" s="94">
         <v>813</v>
       </c>
-      <c r="O34" s="45"/>
-    </row>
-    <row r="35" spans="1:15" ht="55.5" customHeight="1">
+      <c r="O34" s="97">
+        <v>94</v>
+      </c>
+      <c r="P34" s="97"/>
+      <c r="Q34" s="99"/>
+    </row>
+    <row r="35" spans="1:17" ht="55.5" customHeight="1">
       <c r="A35" s="47" t="s">
         <v>2559</v>
       </c>
@@ -31589,12 +31868,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N35" s="47">
+      <c r="N35" s="94">
         <v>813</v>
       </c>
-      <c r="O35" s="45"/>
-    </row>
-    <row r="36" spans="1:15" ht="53.25" customHeight="1">
+      <c r="O35" s="97">
+        <v>151</v>
+      </c>
+      <c r="P35" s="97">
+        <v>294</v>
+      </c>
+      <c r="Q35" s="99"/>
+    </row>
+    <row r="36" spans="1:17" ht="53.25" customHeight="1">
       <c r="A36" s="47" t="s">
         <v>2556</v>
       </c>
@@ -31636,12 +31921,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,p]</v>
       </c>
-      <c r="N36" s="47">
+      <c r="N36" s="94">
         <v>491.20299999999997</v>
       </c>
-      <c r="O36" s="45"/>
-    </row>
-    <row r="37" spans="1:15" ht="43.5" customHeight="1">
+      <c r="O36" s="98" t="s">
+        <v>2795</v>
+      </c>
+      <c r="P36" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q36" s="99"/>
+    </row>
+    <row r="37" spans="1:17" ht="43.5" customHeight="1">
       <c r="A37" s="82" t="s">
         <v>2567</v>
       </c>
@@ -31683,12 +31974,16 @@
         <f t="shared" si="1"/>
         <v>[f,f,n]</v>
       </c>
-      <c r="N37" s="47" t="s">
+      <c r="N37" s="94" t="s">
         <v>2570</v>
       </c>
-      <c r="O37" s="45"/>
-    </row>
-    <row r="38" spans="1:15" ht="38.25" customHeight="1">
+      <c r="O37" s="97">
+        <v>94</v>
+      </c>
+      <c r="P37" s="97"/>
+      <c r="Q37" s="99"/>
+    </row>
+    <row r="38" spans="1:17" ht="38.25" customHeight="1">
       <c r="A38" s="47" t="s">
         <v>2567</v>
       </c>
@@ -31730,12 +32025,18 @@
         <f t="shared" si="1"/>
         <v>[p,p,n]</v>
       </c>
-      <c r="N38" s="47">
+      <c r="N38" s="94">
         <v>707.23800000000006</v>
       </c>
-      <c r="O38" s="45"/>
-    </row>
-    <row r="39" spans="1:15" ht="34.5" customHeight="1">
+      <c r="O38" s="97">
+        <v>151</v>
+      </c>
+      <c r="P38" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q38" s="99"/>
+    </row>
+    <row r="39" spans="1:17" ht="34.5" customHeight="1">
       <c r="A39" s="47" t="s">
         <v>2567</v>
       </c>
@@ -31777,12 +32078,18 @@
         <f t="shared" si="1"/>
         <v>[n,f,f]</v>
       </c>
-      <c r="N39" s="47">
+      <c r="N39" s="94">
         <v>707.23800000000006</v>
       </c>
-      <c r="O39" s="45"/>
-    </row>
-    <row r="40" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O39" s="97">
+        <v>151</v>
+      </c>
+      <c r="P39" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q39" s="99"/>
+    </row>
+    <row r="40" spans="1:17" ht="15.75" customHeight="1">
       <c r="A40" s="47" t="s">
         <v>2567</v>
       </c>
@@ -31824,12 +32131,16 @@
         <f t="shared" si="1"/>
         <v>[f,f,n]</v>
       </c>
-      <c r="N40" s="47">
+      <c r="N40" s="94">
         <v>707.23800000000006</v>
       </c>
-      <c r="O40" s="45"/>
-    </row>
-    <row r="41" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O40" s="97">
+        <v>115</v>
+      </c>
+      <c r="P40" s="97"/>
+      <c r="Q40" s="99"/>
+    </row>
+    <row r="41" spans="1:17" ht="15.75" customHeight="1">
       <c r="A41" s="47" t="s">
         <v>2577</v>
       </c>
@@ -31871,12 +32182,16 @@
         <f t="shared" si="1"/>
         <v>[n,n,p]</v>
       </c>
-      <c r="N41" s="47">
+      <c r="N41" s="94">
         <v>238</v>
       </c>
-      <c r="O41" s="45"/>
-    </row>
-    <row r="42" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O41" s="97">
+        <v>125</v>
+      </c>
+      <c r="P41" s="97"/>
+      <c r="Q41" s="99"/>
+    </row>
+    <row r="42" spans="1:17" ht="42.75" customHeight="1">
       <c r="A42" s="47" t="s">
         <v>2580</v>
       </c>
@@ -31918,12 +32233,18 @@
         <f t="shared" si="1"/>
         <v>[n,n,p]</v>
       </c>
-      <c r="N42" s="47">
+      <c r="N42" s="94">
         <v>119</v>
       </c>
-      <c r="O42" s="45"/>
-    </row>
-    <row r="43" spans="1:15" ht="42.75" customHeight="1">
+      <c r="O42" s="97">
+        <v>125</v>
+      </c>
+      <c r="P42" s="97">
+        <v>488</v>
+      </c>
+      <c r="Q42" s="99"/>
+    </row>
+    <row r="43" spans="1:17" ht="42.75" customHeight="1">
       <c r="A43" s="47" t="s">
         <v>2580</v>
       </c>
@@ -31965,12 +32286,16 @@
         <f t="shared" si="1"/>
         <v>[p,p,n]</v>
       </c>
-      <c r="N43" s="47">
+      <c r="N43" s="94">
         <v>268</v>
       </c>
-      <c r="O43" s="45"/>
-    </row>
-    <row r="44" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O43" s="97">
+        <v>94</v>
+      </c>
+      <c r="P43" s="97"/>
+      <c r="Q43" s="99"/>
+    </row>
+    <row r="44" spans="1:17" ht="15.75" customHeight="1">
       <c r="A44" s="47" t="s">
         <v>2580</v>
       </c>
@@ -32012,12 +32337,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N44" s="47">
+      <c r="N44" s="94">
         <v>119.268</v>
       </c>
-      <c r="O44" s="45"/>
-    </row>
-    <row r="45" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O44" s="97">
+        <v>115</v>
+      </c>
+      <c r="P44" s="97">
+        <v>203</v>
+      </c>
+      <c r="Q44" s="99"/>
+    </row>
+    <row r="45" spans="1:17" ht="15.75" customHeight="1">
       <c r="A45" s="82" t="s">
         <v>2585</v>
       </c>
@@ -32059,12 +32390,18 @@
         <f t="shared" si="1"/>
         <v>[p,n,n]</v>
       </c>
-      <c r="N45" s="47">
+      <c r="N45" s="94">
         <v>172</v>
       </c>
-      <c r="O45" s="45"/>
-    </row>
-    <row r="46" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O45" s="98" t="s">
+        <v>2792</v>
+      </c>
+      <c r="P45" s="97">
+        <v>117</v>
+      </c>
+      <c r="Q45" s="99"/>
+    </row>
+    <row r="46" spans="1:17" ht="15.75" customHeight="1">
       <c r="A46" s="82" t="s">
         <v>2585</v>
       </c>
@@ -32106,12 +32443,18 @@
         <f t="shared" si="1"/>
         <v>[n,n,p]</v>
       </c>
-      <c r="N46" s="47">
+      <c r="N46" s="94">
         <v>172</v>
       </c>
-      <c r="O46" s="45"/>
-    </row>
-    <row r="47" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O46" s="97">
+        <v>125</v>
+      </c>
+      <c r="P46" s="97">
+        <v>488</v>
+      </c>
+      <c r="Q46" s="99"/>
+    </row>
+    <row r="47" spans="1:17" ht="15.75" customHeight="1">
       <c r="A47" s="82" t="s">
         <v>2585</v>
       </c>
@@ -32153,12 +32496,18 @@
         <f t="shared" si="1"/>
         <v>[p,p,n]</v>
       </c>
-      <c r="N47" s="47">
+      <c r="N47" s="94">
         <v>172</v>
       </c>
-      <c r="O47" s="45"/>
-    </row>
-    <row r="48" spans="1:15" ht="15.75" customHeight="1">
+      <c r="O47" s="98" t="s">
+        <v>2795</v>
+      </c>
+      <c r="P47" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q47" s="97"/>
+    </row>
+    <row r="48" spans="1:17" ht="15.75" customHeight="1">
       <c r="A48" s="82" t="s">
         <v>2585</v>
       </c>
@@ -32200,10 +32549,16 @@
         <f t="shared" si="1"/>
         <v>[n,p,n]</v>
       </c>
-      <c r="N48" s="47">
+      <c r="N48" s="94">
         <v>172</v>
       </c>
-      <c r="O48" s="45"/>
+      <c r="O48" s="97">
+        <v>151</v>
+      </c>
+      <c r="P48" s="97">
+        <v>272</v>
+      </c>
+      <c r="Q48" s="97"/>
     </row>
     <row r="49" spans="1:14" ht="15.75" customHeight="1">
       <c r="A49" s="45"/>
@@ -33172,6 +33527,16 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
+  <conditionalFormatting sqref="O1:Q1">
+    <cfRule type="containsBlanks" dxfId="1" priority="2" stopIfTrue="1">
+      <formula>LEN(TRIM(O1))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O2:Q2">
+    <cfRule type="containsBlanks" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>LEN(TRIM(O2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>